<commit_message>
scan: seg0 2026-06-23 01:15 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq1_2026-06-22.xlsx
@@ -538,7 +538,7 @@
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1046.398558076305</v>
+        <v>1026.398558076305</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>52.4</v>
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>63.71081379269862</v>
+        <v>63.71081374237693</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>20.22880587990956</v>
+        <v>20.22880584394183</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.239855807630535</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.6052673331484548</v>
+        <v>0.6052673332926928</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>985.0508296179696</v>
+        <v>1000.05082961797</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>181</v>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>65.18606855667423</v>
+        <v>65.18606851119674</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.01644161156663</v>
+        <v>21.01644159686909</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>0.8252537153339339</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.3937035647726024</v>
+        <v>0.3937035652877401</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>984.2294036338496</v>
+        <v>974.2294036338496</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>56.2</v>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>65.18151091911577</v>
+        <v>65.1815109014611</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>22.54050493798855</v>
+        <v>22.54050492832429</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.8715438144866375</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.5723600297322851</v>
+        <v>0.5723600298044081</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>970.1568755485844</v>
+        <v>960.1568755485844</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>10.15</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>69.71128114912372</v>
+        <v>69.71128110266396</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>21.73816173935355</v>
+        <v>21.73816175939562</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>3.115687554858438</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1637824977929608</v>
+        <v>0.1637824978156277</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>940.4057346256712</v>
+        <v>930.4057346256714</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>152.5</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>79.51327046327535</v>
+        <v>79.51327045652801</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>29.75755822091576</v>
+        <v>29.75755818447251</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0.6668207172621886</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>4.506127460746772</v>
+        <v>4.506127460849804</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>935.3591063422858</v>
+        <v>925.3591063422858</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>12.05</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>65.49773769652045</v>
+        <v>65.49773763611833</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>21.19165318745853</v>
+        <v>21.19165318201537</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.771959847244197</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.110379649517864</v>
+        <v>0.1103796495446519</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>62.18473306379608</v>
+        <v>62.18473305051365</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>44.70759896910476</v>
+        <v>44.70759908190154</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>2.04196008471112</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-0.2582385100799396</v>
+        <v>-0.2582385100181188</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>1342</v>
+        <v>1568</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>八貫</t>
+          <t>倉佑</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>822.5437198628049</v>
+        <v>821.3154059763556</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>117</v>
+        <v>43.3</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,16 +923,16 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>73.50283120017706</v>
+        <v>58.46874764477078</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>43.99316510990627</v>
+        <v>45.70146834435849</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.8119194392723156</v>
+        <v>1.789722097902346</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.251478570677797</v>
+        <v>-0.2713178458846337</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>1568</v>
+        <v>1342</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>倉佑</t>
+          <t>八貫</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>821.3154059763556</v>
+        <v>812.5437198628049</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>43.3</v>
+        <v>117</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,16 +976,16 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>58.46874766623961</v>
+        <v>73.5028311573335</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>45.70146829859155</v>
+        <v>43.99316514393011</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.789722097902346</v>
+        <v>0.8119194392723156</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
@@ -994,11 +994,11 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.2713178459979684</v>
+        <v>1.251478571028093</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>68.82540958222789</v>
+        <v>68.82540949283295</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>31.18532568871135</v>
+        <v>31.1853257203507</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.6889538191076813</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.2262549132958999</v>
+        <v>0.2262549136668086</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64.59551279932063</v>
+        <v>64.59551262388973</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>26.11347915471536</v>
+        <v>26.11347920994383</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.463881395452544</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.09320498960285251</v>
+        <v>0.0932049896543702</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>769.3672423803047</v>
+        <v>769.3672423803046</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>54.7</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>56.00850879689729</v>
+        <v>56.00850929820249</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>28.35870239877566</v>
+        <v>28.35870258041111</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.2875217889101</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.0708883844313843</v>
+        <v>0.0708883839986641</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>748.6320237460199</v>
+        <v>748.6320237460197</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>713</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>58.40469152839113</v>
+        <v>58.40469148272824</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>23.15434142865251</v>
+        <v>23.1543412931821</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.096035889670256</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-2.414808132909343</v>
+        <v>-2.414808128376052</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>69.911045073276</v>
+        <v>69.9110450800742</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>25.71180094611355</v>
+        <v>25.71180092700941</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.458850610405508</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.3684339379689705</v>
+        <v>0.3684339380204817</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>62.99190918703215</v>
+        <v>62.99190914103388</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>21.31109670360736</v>
+        <v>21.31109667936443</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.7800091683492597</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.6568076319510112</v>
+        <v>0.6568076327752532</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>72.50230117383245</v>
+        <v>72.5023011299548</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>23.46369920573198</v>
+        <v>23.46369943417819</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.338622358203861</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.2309578191467627</v>
+        <v>0.2309578192497899</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>722.7769534139868</v>
+        <v>712.7769534139868</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>8.039999999999999</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>60.34134175882714</v>
+        <v>60.34134174082925</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>15.946604728466</v>
+        <v>15.94660470911001</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.169985738879141</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.0172045437095062</v>
+        <v>0.0172045437177483</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>72.43416232315207</v>
+        <v>72.43416227967579</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.62581181699131</v>
+        <v>23.62581182450628</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>3.795549731476423</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.0897190527090489</v>
+        <v>0.0897190527296533</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>65.32159720691902</v>
+        <v>65.32159720378715</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>32.91816200912373</v>
+        <v>32.91816197901861</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.409317206060858</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-0.008357900603189</v>
+        <v>-0.0083579005825837</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>52.52155100671608</v>
+        <v>52.52155100946299</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>12.20294098382363</v>
+        <v>12.20294097485596</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>5.040319454136621</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.5251358932892181</v>
+        <v>-0.5251358934231556</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>62.74158512706924</v>
+        <v>62.74158505338232</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>30.28540804498776</v>
+        <v>30.28540809085413</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.11035896961442</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.0767802848240732</v>
+        <v>0.07678028488589179</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>679.4069826835847</v>
+        <v>679.4069826835848</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>74.3</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>52.12272212005704</v>
+        <v>52.12272213422671</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>20.7127896872034</v>
+        <v>20.71278977343094</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.8324820287392075</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.037695472163985</v>
+        <v>0.0376954721433906</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1693,21 +1693,21 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>1514</v>
+        <v>1338</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>亞力</t>
+          <t>廣華-KY</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>670.7868478514449</v>
+        <v>664.8921902511222</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>127</v>
+        <v>17.2</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>54.85542293878647</v>
+        <v>60.37026792704671</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>22.82464164063456</v>
+        <v>21.87266943551693</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1.466760654491019</v>
+        <v>0.3679077906811365</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.7894858860542115</v>
+        <v>0.0591816415692871</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>1338</v>
+        <v>1102</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>廣華-KY</t>
+          <t>亞泥</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>664.8921902511222</v>
+        <v>652.8175225126929</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>17.2</v>
+        <v>36.35</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>60.37026801445862</v>
+        <v>67.47554745417354</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>21.87266924133029</v>
+        <v>17.60717112700948</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.3679077906811365</v>
+        <v>0.7278136103204178</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.0591816414765631</v>
+        <v>0.2715096534883743</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>1102</v>
+        <v>1236</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>亞泥</t>
+          <t>宏亞</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>652.8175225126929</v>
+        <v>652.5483124744744</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>36.35</v>
+        <v>25.85</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>67.47554746911665</v>
+        <v>64.13107347497127</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>17.6071711245829</v>
+        <v>14.94042744061894</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.7278136103204178</v>
+        <v>1.354831247447447</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.2715096534368624</v>
+        <v>0.106203334472837</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>1236</v>
+        <v>1514</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>宏亞</t>
+          <t>亞力</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>652.5483124744744</v>
+        <v>650.7868478514451</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>25.85</v>
+        <v>127</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,16 +1877,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>64.13107895877562</v>
+        <v>54.85542288888971</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>14.94042919156888</v>
+        <v>22.82464163553545</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1.354831247447447</v>
+        <v>1.466760654491019</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.1062033301353141</v>
+        <v>-0.7894858854154281</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>1443</v>
+        <v>1532</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>立益</t>
+          <t>勤美</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>618.708268680246</v>
+        <v>583.026265524765</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>27.45</v>
+        <v>23.3</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>61.23749848990025</v>
+        <v>61.11492663311383</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>20.14507788557326</v>
+        <v>39.81838907859251</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.4493460019743336</v>
+        <v>0.9625296764123976</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0980499996891495</v>
+        <v>0.1538957504276021</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>1532</v>
+        <v>1110</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>勤美</t>
+          <t>東泥</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>583.026265524765</v>
+        <v>581.4780629556602</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>23.3</v>
+        <v>15.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>61.11492664591576</v>
+        <v>56.02365821237996</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>39.81838896452918</v>
+        <v>32.98570957805581</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.9625296764123976</v>
+        <v>0.4387359657660677</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.1538957503657833</v>
+        <v>0.0381243831210871</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2011,21 +2011,21 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>1110</v>
+        <v>1437</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>東泥</t>
+          <t>勤益控</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>581.4780629556602</v>
+        <v>577.8873412787611</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>15.5</v>
+        <v>29.75</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>56.02365831719868</v>
+        <v>63.28144592145673</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>32.98570925093466</v>
+        <v>26.8492911597504</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.4387359657660677</v>
+        <v>0.9905425967234426</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.0381243830077543</v>
+        <v>0.1435010032716756</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>1437</v>
+        <v>1446</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>勤益控</t>
+          <t>宏和</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>577.8873412787617</v>
+        <v>576.784029086406</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>29.75</v>
+        <v>16.55</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>63.28144605471008</v>
+        <v>55.62541636291561</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.84929109736101</v>
+        <v>26.00301781406289</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.9905425967234426</v>
+        <v>1.002787881922972</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1435010032201613</v>
+        <v>0.0153111533343068</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>1446</v>
+        <v>1455</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>宏和</t>
+          <t>集盛</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>576.784029086406</v>
+        <v>572.0016556668469</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>16.55</v>
+        <v>9.76</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>55.62541658556755</v>
+        <v>60.12642985436876</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>26.00301780312343</v>
+        <v>43.77281169494158</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.002787881922972</v>
+        <v>1.213574897917097</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.0153111532312757</v>
+        <v>0.0306375276058465</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>1455</v>
+        <v>1414</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>集盛</t>
+          <t>東和</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>572.0016556668469</v>
+        <v>569.9924782353484</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>9.76</v>
+        <v>17.55</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>60.12642985908226</v>
+        <v>65.29761603441636</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>43.77281155227252</v>
+        <v>25.58017478249677</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.213574897917097</v>
+        <v>0.439903845187051</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.0306375275914231</v>
+        <v>0.1762494480607601</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>1414</v>
+        <v>1443</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>東和</t>
+          <t>立益</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>569.992478235348</v>
+        <v>558.7082686802461</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>17.55</v>
+        <v>27.45</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>65.29761628542482</v>
+        <v>61.23749554020946</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>25.58017462177521</v>
+        <v>20.14507630583234</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.439903845187051</v>
+        <v>0.4493460019743336</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.1762494477958988</v>
+        <v>0.098050005541193</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>1304</v>
+        <v>1504</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>台聚</t>
+          <t>東元</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>547.1394715146919</v>
+        <v>546.6612204990133</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>13.7</v>
+        <v>72.2</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>58.39021048491747</v>
+        <v>50.42629732331334</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>18.57345407609298</v>
+        <v>21.09645082999722</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.189369052399414</v>
+        <v>0.3734186532931434</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.1227590158071714</v>
+        <v>-0.7515562723727779</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>1504</v>
+        <v>1525</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>東元</t>
+          <t>江申</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>546.6612204990133</v>
+        <v>540.3130271354463</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>72.2</v>
+        <v>66</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>50.42629733967912</v>
+        <v>51.98658026033768</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>21.09645084641164</v>
+        <v>28.01255592810987</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.3734186532931434</v>
+        <v>0.2053491987654774</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>1</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.7515562725170363</v>
+        <v>-0.3779477529698274</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>1525</v>
+        <v>1308</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>江申</t>
+          <t>亞聚</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>540.3130271354463</v>
+        <v>539.8656565567961</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>66</v>
+        <v>14.15</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>51.98658032645178</v>
+        <v>56.53953509452306</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>28.01255593262242</v>
+        <v>15.44683890935274</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.2053491987654774</v>
+        <v>0.9612350327228468</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.3779477529286226</v>
+        <v>0.1095707365833335</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>1308</v>
+        <v>1535</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>亞聚</t>
+          <t>中宇</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>539.8656565567961</v>
+        <v>539.6570868060044</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>14.15</v>
+        <v>50.3</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>56.53953519515458</v>
+        <v>51.81308255664876</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>15.44683889318586</v>
+        <v>25.37440883099461</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.9612350327228468</v>
+        <v>1.504159064655777</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.1095707365730296</v>
+        <v>0.0800496390124308</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>1535</v>
+        <v>1444</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>中宇</t>
+          <t>力麗</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>539.6570868060044</v>
+        <v>538.4426676289412</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>50.3</v>
+        <v>7.01</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>51.8130826668764</v>
+        <v>57.96496817217107</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>25.37440874823943</v>
+        <v>32.90460091667379</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.504159064655777</v>
+        <v>0.5915648153609725</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.08004963882697939</v>
+        <v>0.0009049487127112</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>1444</v>
+        <v>1304</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>力麗</t>
+          <t>台聚</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>538.4426676289412</v>
+        <v>537.1394715146919</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>7.01</v>
+        <v>13.7</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>57.96496819057322</v>
+        <v>58.39021040346858</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>32.90460081146784</v>
+        <v>18.5734541319836</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.5915648153609725</v>
+        <v>1.189369052399414</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,11 +2584,11 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.0009049486962265</v>
+        <v>0.1227590158483827</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>54.34590162291522</v>
+        <v>54.34590183155601</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>48.26193628708469</v>
+        <v>48.26193620399269</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.4553976256472893</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.3104675181762502</v>
+        <v>-0.3104675181144274</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>45.44859861151803</v>
+        <v>45.44859862757233</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>27.62529823001249</v>
+        <v>27.62529825702557</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.5170782096367672</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.4289648755174841</v>
+        <v>-0.4289648755277913</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>55.53043168086514</v>
+        <v>55.53043161058248</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>23.04658500975085</v>
+        <v>23.04658508041436</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.3558363494559451</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.0229322269689442</v>
+        <v>-0.0229322269277322</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>55.58604574011583</v>
+        <v>55.5860456477355</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>12.59012015976604</v>
+        <v>12.5901202116165</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.8669118505809028</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1195938797766635</v>
+        <v>0.1195938798178744</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>508.2278547177094</v>
+        <v>508.2278547177096</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>12.9</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>54.89292340131996</v>
+        <v>54.89292335344354</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>18.81736756251582</v>
+        <v>18.81736752740409</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.3244639492867056</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.0282771342546074</v>
+        <v>0.0282771342958185</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>56.34915870024526</v>
+        <v>56.34915871475492</v>
       </c>
       <c r="I46" s="2" t="n">
         <v>43.84271006154518</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.2970826830128413</v>
+        <v>0.2970826829510211</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>59.04749020588115</v>
+        <v>59.04748998982353</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>30.20649792265771</v>
+        <v>30.20649799616193</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>2.497422011506554</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.0518463153467999</v>
+        <v>0.0518463154086152</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>486.359171486863</v>
+        <v>486.3591714868634</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>66.2</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>53.43818053457659</v>
+        <v>53.43818050546939</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>21.30717517833261</v>
+        <v>21.30717520014517</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.115187532371392</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.06652675978917121</v>
+        <v>0.0665267598200789</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>51.5031018659784</v>
+        <v>51.50310179381555</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>14.18415714106323</v>
+        <v>14.18415721810027</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1.035329906302542</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.0014680785106931</v>
+        <v>0.0014680785189343</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>51.27888318713648</v>
+        <v>51.27888300669188</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>27.6277008344214</v>
+        <v>27.6277013226409</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.688838301202248</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0007682189192813</v>
+        <v>-0.0007682188574642</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>46.21780666316818</v>
+        <v>46.21780666748565</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.598397457486463</v>
+        <v>8.598397412560191</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.3755606533315579</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.1557135209619244</v>
+        <v>-0.1557135208485953</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>54.16001267017564</v>
+        <v>54.16001235446382</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>21.08764196890775</v>
+        <v>21.08764204495171</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.6772631704487966</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.2120016621500803</v>
+        <v>0.2120016622943213</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>60.1417335754652</v>
+        <v>60.14173343396394</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>15.70078549719329</v>
+        <v>15.70078557689049</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.9553472393181071</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0491192718921317</v>
+        <v>0.0491192719127386</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>29.84417130225067</v>
+        <v>29.8441713475388</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>28.64542881557074</v>
+        <v>28.6454287754692</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.162975976898777</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.5021190472834658</v>
+        <v>-0.5021190473040734</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.21704238197474</v>
+        <v>44.21704221071857</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>21.70269556375217</v>
+        <v>21.70269559806124</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.8991257047605385</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0457005808853042</v>
+        <v>0.0457005809574218</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>62.57060614641512</v>
+        <v>62.57060617502798</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>18.51539503356821</v>
+        <v>18.51539508448864</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.4233188339001434</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.2202050906869305</v>
+        <v>0.2202050906972319</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3495,21 +3495,21 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>1477</v>
+        <v>1524</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>聚陽</t>
+          <t>耿鼎</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>455.5189925524314</v>
+        <v>452.7434026728614</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>213.5</v>
+        <v>29.7</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>41.25321944763096</v>
+        <v>46.5926826735509</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.67392719562585</v>
+        <v>15.23229736270177</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>2.019816030076471</v>
+        <v>0.3222458277424332</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.6908548407903702</v>
+        <v>-0.2668152081881562</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>1524</v>
+        <v>1436</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>耿鼎</t>
+          <t>華友聯</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>452.7434026728615</v>
+        <v>448.5206740453645</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>29.7</v>
+        <v>45.7</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>46.5926828079992</v>
+        <v>45.29824907114076</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>15.23229705100422</v>
+        <v>28.41713388184188</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.3222458277424332</v>
+        <v>1.78375206019303</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.2668152083942142</v>
+        <v>0.3152691464632978</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>1436</v>
+        <v>1477</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>華友聯</t>
+          <t>聚陽</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>448.5206740453645</v>
+        <v>445.5189925524314</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>45.7</v>
+        <v>213.5</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>45.2982491122081</v>
+        <v>41.25321937881883</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>28.41713387532161</v>
+        <v>23.67392722802721</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.78375206019303</v>
+        <v>2.019816030076471</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,11 +3644,11 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.3152691463602702</v>
+        <v>-0.6908548402752441</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>56.73017836529714</v>
+        <v>56.73017820734288</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>18.7827299945112</v>
+        <v>18.78273018943973</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.4047307774091722</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.1114217892532211</v>
+        <v>0.1114217892944328</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.92307407339477</v>
+        <v>49.92307404232423</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>29.14969660459841</v>
+        <v>29.14969652827201</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.5416381688928046</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.0851466524432398</v>
+        <v>-0.0851466524329369</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3760,21 +3760,21 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>1319</v>
+        <v>1217</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>東陽</t>
+          <t>愛之味</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>424.218517999157</v>
+        <v>418.8364300207993</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>84.8</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>42.11810615061632</v>
+        <v>56.04288189763709</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>34.39360504170578</v>
+        <v>21.78008981619977</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>2.256930517199805</v>
+        <v>0.6638187341726167</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-1.14352864338175</v>
+        <v>0.0140759726233061</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>1217</v>
+        <v>1323</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>愛之味</t>
+          <t>永裕</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>418.8364300207993</v>
+        <v>418.7705850502326</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>9.890000000000001</v>
+        <v>20</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>56.04288182800006</v>
+        <v>50.49423753375167</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>21.78008978353489</v>
+        <v>15.18736836009719</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.6638187341726167</v>
+        <v>4.021516365077394</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.0140759726336092</v>
+        <v>-0.0016939378123344</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>1323</v>
+        <v>1229</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>永裕</t>
+          <t>聯華</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>418.7705850502326</v>
+        <v>415.899290946783</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>20</v>
+        <v>41.2</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>50.49423741970813</v>
+        <v>48.38491989163624</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>15.18736834668963</v>
+        <v>24.19483307769558</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>4.021516365077394</v>
+        <v>0.8747980928893067</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.00169393777112</v>
+        <v>0.0573471516317109</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>1229</v>
+        <v>1442</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>聯華</t>
+          <t>名軒</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>415.899290946783</v>
+        <v>415.1546995641552</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>41.2</v>
+        <v>27.4</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>48.38491994192729</v>
+        <v>51.9896487471243</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>24.19483315330073</v>
+        <v>21.83636740565806</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.8747980928893067</v>
+        <v>0.7240854146990087</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0573471515595935</v>
+        <v>0.0904234388821941</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>1442</v>
+        <v>1537</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>名軒</t>
+          <t>廣隆</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>415.1546995641552</v>
+        <v>415.0647768396969</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>27.4</v>
+        <v>127</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>51.98964858090528</v>
+        <v>54.96443574236747</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>21.83636749881414</v>
+        <v>10.06409097725938</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.7240854146990087</v>
+        <v>0.6731826022390055</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.09042343894401041</v>
+        <v>-0.0437120093000305</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>1537</v>
+        <v>1319</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>廣隆</t>
+          <t>東陽</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>415.0647768396969</v>
+        <v>414.218517999157</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>127</v>
+        <v>84.8</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>54.96443582725154</v>
+        <v>42.11810604341566</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>10.06409087358666</v>
+        <v>34.39360508750283</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.6731826022390055</v>
+        <v>2.256930517199805</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>1</v>
@@ -4068,11 +4068,11 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.0437120095061013</v>
+        <v>-1.14352864235147</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>54.18198298129921</v>
+        <v>54.18198299040751</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>13.75545317008814</v>
+        <v>13.75545313865143</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.37064243209637</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0375951319028562</v>
+        <v>0.0375951322943661</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>1466</v>
+        <v>1315</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>聚隆</t>
+          <t>達新</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>412.8768050633577</v>
+        <v>410.4901627602394</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>14.65</v>
+        <v>62.2</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>50.43273214171141</v>
+        <v>55.36834163429479</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>16.44486688454207</v>
+        <v>12.91255415298573</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.8876805063357643</v>
+        <v>0.8414417205270101</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0813594136695751</v>
+        <v>0.1295553738279113</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>1315</v>
+        <v>1521</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>達新</t>
+          <t>大億</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>410.4901627602393</v>
+        <v>405.9853802052307</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>62.2</v>
+        <v>26.55</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>55.36834170615894</v>
+        <v>53.75815423875723</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>12.91255424160086</v>
+        <v>19.99965760573953</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.8414417205270101</v>
+        <v>0.3785933421877506</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1295553738485124</v>
+        <v>-0.0848889940249714</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, cci_momentum</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>1521</v>
+        <v>1466</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>大億</t>
+          <t>聚隆</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>405.9853802052306</v>
+        <v>402.8768050633577</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>26.55</v>
+        <v>14.65</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>53.75815430852412</v>
+        <v>50.43273215265129</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>19.99965753177656</v>
+        <v>16.44486692732539</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.3785933421877506</v>
+        <v>0.8876805063357643</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,11 +4280,11 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0848889940146698</v>
+        <v>0.08135941357684939</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>49.49447322008906</v>
+        <v>49.49447332244184</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>10.78289487652052</v>
+        <v>10.78289492074228</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>3.768135583011466</v>
@@ -4343,21 +4343,21 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>1309</v>
+        <v>1203</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>台達化</t>
+          <t>味王</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>390.7192609400598</v>
+        <v>387.1341085927021</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>15.05</v>
+        <v>42.8</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,16 +4368,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>43.10832256378383</v>
+        <v>49.81007716586731</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>11.36289588409538</v>
+        <v>17.86574023003663</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.6363686568049091</v>
+        <v>0.5168396253716593</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0104967974695261</v>
+        <v>-0.0156046123021651</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>1203</v>
+        <v>1256</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>味王</t>
+          <t>鮮活果汁-KY</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>387.1341085927021</v>
+        <v>385.8871427485622</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>42.8</v>
+        <v>181</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>49.81007715909335</v>
+        <v>48.76698112757373</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>17.86574021781098</v>
+        <v>20.84600926398029</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.5168396253716593</v>
+        <v>0.2073958893580916</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.0156046122815594</v>
+        <v>-1.829568909851212</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>1256</v>
+        <v>1453</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>鮮活果汁-KY</t>
+          <t>大將</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>385.8871427485622</v>
+        <v>383.5614318001943</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>181</v>
+        <v>11.65</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>48.76698122868041</v>
+        <v>52.52231077389309</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>20.84600950606863</v>
+        <v>28.54067303116454</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.2073958893580916</v>
+        <v>0.5097541525352729</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-1.8295689109845</v>
+        <v>0.0624784771276745</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>1453</v>
+        <v>1309</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>大將</t>
+          <t>台達化</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>383.5614318001944</v>
+        <v>380.7192609400598</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>11.65</v>
+        <v>15.05</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.52231104133784</v>
+        <v>43.10832251966274</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>28.54067297766962</v>
+        <v>11.36289587086999</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.5097541525352729</v>
+        <v>0.6363686568049091</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,11 +4545,11 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0624784770658575</v>
+        <v>0.0104967975210382</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive</t>
         </is>
       </c>
     </row>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>51.45395572357079</v>
+        <v>51.45395561592931</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>24.25945511936088</v>
+        <v>24.25945547314785</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.901808570067641</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.0399388166713361</v>
+        <v>0.0399388167022446</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>53.13293404570278</v>
+        <v>53.13293384970808</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7.999634616147781</v>
+        <v>7.99963467487359</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.2737265170660414</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.5872335185214108</v>
+        <v>0.5872335231165995</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>39.07167603965878</v>
+        <v>39.07167619904473</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>28.33217181753086</v>
+        <v>28.33217186791484</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>1.017408134418036</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0268065630643023</v>
+        <v>0.0268065630849079</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>363.1230906343469</v>
+        <v>363.123090634347</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>10.5</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>54.06668944031902</v>
+        <v>54.06668939549615</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>22.01703156214709</v>
+        <v>22.01703165803896</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>1.403098500267817</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0449732773507291</v>
+        <v>0.0449732773610308</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>362.9310362582885</v>
+        <v>362.9310362582886</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>20.4</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>43.04274032588755</v>
+        <v>43.04274013065121</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>16.08792693345491</v>
+        <v>16.08792693136532</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.2192910853345947</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.08639377218692131</v>
+        <v>-0.08639377201176809</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>361.8459689780391</v>
+        <v>361.845968978039</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>33.1</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>50.56069142052397</v>
+        <v>50.56069125599162</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>17.93086340258118</v>
+        <v>17.9308633806529</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.7810201082984269</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.0214980305624228</v>
+        <v>-0.0214980304800008</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>355.7989143950047</v>
+        <v>345.7989143950047</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>43.6</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>52.77136119530726</v>
+        <v>52.77136105513618</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>23.96415611411509</v>
+        <v>23.96415614471187</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.7151933932497501</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0812434647468088</v>
+        <v>-0.081243464623173</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>336.5929956685446</v>
+        <v>336.5929956685448</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>12.95</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>49.60645366288907</v>
+        <v>49.60645360756141</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>23.61509795205323</v>
+        <v>23.61509795205322</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.2788597055199956</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0129665618741925</v>
+        <v>0.0129665619051031</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>336.5454752145212</v>
+        <v>336.5454752145211</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>12.4</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>52.73024591377889</v>
+        <v>52.7302459799669</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>13.47546987880226</v>
+        <v>13.47546992043969</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.9485964802925472</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0055970433451382</v>
+        <v>0.0055970433142297</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.56389189122566</v>
+        <v>48.56389182422849</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>15.76700814295951</v>
+        <v>15.76700809507664</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.7791134424489916</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.0251182210245043</v>
+        <v>0.0251182210471693</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>331.2926468128384</v>
+        <v>331.2926468128385</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>31.35</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>49.53575847881361</v>
+        <v>49.53575835999958</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>15.79578383307749</v>
+        <v>15.79578389290244</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.5910928023816721</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0490293678495477</v>
+        <v>0.049029368045305</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>328.4570093149432</v>
+        <v>328.457009314943</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>22</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>52.93331937179638</v>
+        <v>52.93331938876045</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>14.92116571386668</v>
+        <v>14.92116570662975</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.9834813217425854</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0236207020227578</v>
+        <v>-0.0236207017548807</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
         <v>49.31067553817468</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>14.44395379346226</v>
+        <v>14.44395375829432</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.142993070591494</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0320777885776626</v>
+        <v>0.0320777886085724</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5244,21 +5244,21 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>1108</v>
+        <v>1476</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>幸福</t>
+          <t>儒鴻</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>298.016073074945</v>
+        <v>305.835234901146</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>13.9</v>
+        <v>317</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,49 +5269,49 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>49.84830145006896</v>
+        <v>36.05380728348681</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>29.86974860453543</v>
+        <v>14.86256861940944</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.246281066402242</v>
+        <v>1.240410845788054</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M91" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.0514694695953752</v>
+        <v>-3.253446988522722</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>1472</v>
+        <v>1108</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>三洋實業</t>
+          <t>幸福</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>297.1162749483781</v>
+        <v>298.016073074945</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>88.59999999999999</v>
+        <v>13.9</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>49.82712634371573</v>
+        <v>49.84830130994358</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>8.798095379682099</v>
+        <v>29.86974875737875</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.3116274948378036</v>
+        <v>1.246281066402242</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>1</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.2475339015009967</v>
+        <v>0.0514694696262838</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>1582</v>
+        <v>1472</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>信錦</t>
+          <t>三洋實業</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>296.0598158195962</v>
+        <v>297.1162749483781</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>93.90000000000001</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>44.36412259307497</v>
+        <v>49.82712612605116</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>20.4417942961077</v>
+        <v>8.79809546145513</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.423465146115219</v>
+        <v>0.3116274948378036</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>1</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-1.415464417491263</v>
+        <v>0.2475339027373525</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>1529</v>
+        <v>1582</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>樂事綠能</t>
+          <t>信錦</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>291.6143316159923</v>
+        <v>296.0598158195962</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>22.7</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>50.75559810995097</v>
+        <v>44.36412254587624</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>17.73029960956027</v>
+        <v>20.44179443866988</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.9008556991250368</v>
+        <v>0.423465146115219</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0237453801812989</v>
+        <v>-1.415464417202782</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>1476</v>
+        <v>1232</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>儒鴻</t>
+          <t>大統益</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>290.8352349011456</v>
+        <v>290.6269326774683</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>317</v>
+        <v>142</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,49 +5481,49 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>36.05380721967424</v>
+        <v>28.24584006570528</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.86256861107685</v>
+        <v>25.49071256778552</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>1.240410845788054</v>
+        <v>1.962693267746835</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M95" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-3.253446990377215</v>
+        <v>-0.6980600315322397</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>1232</v>
+        <v>1413</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>大統益</t>
+          <t>宏洲</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>290.6269326774683</v>
+        <v>290.3763998935169</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>142</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>28.24584008245638</v>
+        <v>48.11195101302914</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>25.49071262701101</v>
+        <v>7.199776996784793</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>1.962693267746835</v>
+        <v>0.613069992134477</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.6980600315322397</v>
+        <v>-0.0161601301491096</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>1413</v>
+        <v>1506</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>宏洲</t>
+          <t>正道</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>290.3763998935168</v>
+        <v>289.6434583933053</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>9.380000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>48.11195103098987</v>
+        <v>45.91553225474299</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>7.199776958981008</v>
+        <v>26.68601425027678</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.613069992134477</v>
+        <v>0.7308698943157692</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.0161601301800192</v>
+        <v>0.0373320739340507</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>1506</v>
+        <v>1438</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>正道</t>
+          <t>三地開發</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>289.6434583933053</v>
+        <v>288.5270114337659</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>10.2</v>
+        <v>21.15</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>45.91553225474299</v>
+        <v>45.40184065113316</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>26.68601420574816</v>
+        <v>26.82443654978456</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.7308698943157692</v>
+        <v>0.9779379614345816</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.0373320739031416</v>
+        <v>0.2630674799730477</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5668,21 +5668,21 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>1438</v>
+        <v>1220</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>三地開發</t>
+          <t>台榮</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>288.5270114337659</v>
+        <v>288.3081927026621</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>21.15</v>
+        <v>11.7</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>45.40184062618933</v>
+        <v>38.38382357076729</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>26.82443648018478</v>
+        <v>29.47119181568361</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.9779379614345816</v>
+        <v>0.7243587334001763</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.2630674799627427</v>
+        <v>0.0199596563995495</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5721,21 +5721,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>1220</v>
+        <v>1467</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>台榮</t>
+          <t>南緯</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>288.3081927026621</v>
+        <v>287.8245296426698</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>11.7</v>
+        <v>7.15</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.38382357076729</v>
+        <v>42.39507528164541</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>29.47119163013281</v>
+        <v>27.67580639169674</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.7243587334001763</v>
+        <v>1.390998209022112</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.0199596563686424</v>
+        <v>-0.0493752826024842</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5774,21 +5774,21 @@
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>1467</v>
+        <v>1410</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>南緯</t>
+          <t>南染</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>287.8245296426698</v>
+        <v>285.3615676987631</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>7.15</v>
+        <v>24.7</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.39507538618015</v>
+        <v>33.02513070287431</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>27.67580631418285</v>
+        <v>15.65975273286436</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>1.390998209022112</v>
+        <v>1.956312668882259</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0493752826169072</v>
+        <v>0.0344647963096695</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>1410</v>
+        <v>1538</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>南染</t>
+          <t>正峰</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>285.3615676987631</v>
+        <v>283.0229349867409</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>24.7</v>
+        <v>11.4</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>33.02513076316302</v>
+        <v>51.39659729746658</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>15.65975272901867</v>
+        <v>6.100783578008504</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.956312668882259</v>
+        <v>1.463889141712933</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0344647962581541</v>
+        <v>-0.2353077384343593</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>1538</v>
+        <v>1519</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>正峰</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>283.0229349867409</v>
+        <v>282.8905227399443</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>11.4</v>
+        <v>831</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>51.39659729746658</v>
+        <v>49.51181979334314</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>6.100783606599332</v>
+        <v>11.04340921734913</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>1.463889141712933</v>
+        <v>0.4067498747327872</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.2353077384343593</v>
+        <v>-0.241491211452999</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>1519</v>
+        <v>1529</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>華城</t>
+          <t>樂事綠能</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>282.8905227399445</v>
+        <v>281.6143316159922</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>831</v>
+        <v>22.7</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>49.511819846629</v>
+        <v>50.75559802985981</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>11.0434093131264</v>
+        <v>17.73029968991498</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.4067498747327872</v>
+        <v>0.9008556991250368</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,11 +5976,11 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.2414912154711768</v>
+        <v>0.0237453802534186</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, dealer_buy_3d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>51.33744044036713</v>
+        <v>51.33744034303702</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>13.11727067582911</v>
+        <v>13.11727066553205</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.269500393157467</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0950926646838694</v>
+        <v>0.0950926648281079</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>31.35571839539389</v>
+        <v>31.35571844745949</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>42.75758736139019</v>
+        <v>42.75758736570336</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.2488381207295223</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.2242677432111453</v>
+        <v>0.2242677430875197</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>34.01915478026007</v>
+        <v>34.01915481121893</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>20.91035807655533</v>
+        <v>20.9103581151721</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.935007787892845</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0402152585850456</v>
+        <v>-0.0402152585232285</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>42.2453865118605</v>
+        <v>42.24538652069045</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>23.70760710370353</v>
+        <v>23.70760716696331</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.7560760053026956</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0418338954911605</v>
+        <v>-0.0418338955426725</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>278.2812298698271</v>
+        <v>278.281229869827</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>8.43</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>47.65506634237963</v>
+        <v>47.655066294748</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>17.12103757642057</v>
+        <v>17.12103762838812</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.093192279590471</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0287581637313399</v>
+        <v>0.0287581637437032</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>276.5365412843663</v>
+        <v>276.5365412843664</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>6.93</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>47.06028339842157</v>
+        <v>47.06028334630847</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>10.61017132401736</v>
+        <v>10.61017135594212</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.215701624530379</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0312468976953691</v>
+        <v>0.0312468977015508</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>41.36216321744404</v>
+        <v>41.36216315010784</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>24.83797795787637</v>
+        <v>24.83797799241428</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>1.581230857192726</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.027661313222513</v>
+        <v>-0.0276613132019068</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>273.0799649972621</v>
+        <v>273.079964997262</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>11.7</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>47.85791605617816</v>
+        <v>47.85791503465682</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.80347279790935</v>
+        <v>14.8034722568372</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>2.434380210448768</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0111710113413467</v>
+        <v>0.0111710115474045</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>48.45064620163627</v>
+        <v>48.45064609515811</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>19.63532893365718</v>
+        <v>19.63532895265388</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.8984446033617258</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>48.64301753482898</v>
+        <v>48.64301747906084</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>21.68483739501346</v>
+        <v>21.68483746585004</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.7277847962805658</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0076268286504022</v>
+        <v>0.0076268286710081</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>45.10245049393343</v>
+        <v>45.10245036557522</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>21.29412638170665</v>
+        <v>21.29412648302154</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.003902103125874</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0208103070841689</v>
+        <v>-0.0208103070635627</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>50.56888498956919</v>
+        <v>50.5688849770286</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>10.7523833038152</v>
+        <v>10.75238333136414</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>6.697354771784233</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.1375161651027481</v>
+        <v>0.1375161651542621</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>50.42794597376307</v>
+        <v>50.427946101083</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>14.01562480668248</v>
+        <v>14.01562486931417</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.6578041512190774</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.020346528527113</v>
+        <v>0.0203465285538989</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>37.06904271266575</v>
+        <v>37.06904253816798</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.9182499150426</v>
+        <v>23.91825026864246</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>1.323710396850224</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0143822765279992</v>
+        <v>0.0143822765795126</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>44.56797362512447</v>
+        <v>44.56797363256914</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>5.526636462539425</v>
+        <v>5.526636413705717</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>1.081993793413859</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0602561240132501</v>
+        <v>-0.0602561240235519</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>205.244530879015</v>
+        <v>205.2445308790182</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>17.45</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>37.52439557271062</v>
+        <v>37.52439453308263</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>13.18177448745928</v>
+        <v>13.18177530871912</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1.229990146256363</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0095051170419555</v>
+        <v>-0.0095051167431711</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>39.66183978234042</v>
+        <v>39.66184046024319</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>15.77498136370684</v>
+        <v>15.77498124757377</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>2.144893385318134</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>29.58059606728517</v>
+        <v>29.58059600077931</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>29.37748317021224</v>
+        <v>29.37748319861415</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.6358573526377318</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.1565167956065248</v>
+        <v>-0.1565167955859193</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>50.61040846053511</v>
+        <v>50.61040840445925</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>18.2645306793833</v>
+        <v>18.26453065329736</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>1.220386585503557</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0514527154329735</v>
+        <v>0.0514527154432762</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>194.5986834939918</v>
+        <v>194.5986834939919</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>10.5</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>44.40601393612649</v>
+        <v>44.40601378150549</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>19.21776004149869</v>
+        <v>19.21776008727772</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>1.030269035192337</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0592389933185207</v>
+        <v>0.0592389933803368</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>186.5716576346476</v>
+        <v>186.5716576346473</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>10.7</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>26.27476558727069</v>
+        <v>26.27476529337858</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.3633723442537</v>
+        <v>17.36337239035742</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>2.863845135044508</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.026286480637237</v>
+        <v>-0.0262864805445112</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>174.5455346758892</v>
+        <v>174.5455346758891</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>14.2</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>43.42397148361876</v>
+        <v>43.4239713972396</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>19.04779787482895</v>
+        <v>19.0477980291148</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.523915980302436</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.030594773028412</v>
+        <v>-0.030594772997502</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>40.87812780535857</v>
+        <v>40.87812769366802</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>14.42880514179021</v>
+        <v>14.42880513743369</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.9011069695876724</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0525096195167968</v>
+        <v>-0.0525096190325635</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>38.80765388204609</v>
+        <v>38.8076543557684</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>13.34074816505444</v>
+        <v>13.34074817284156</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>1.483011223514017</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.0718991442980043</v>
+        <v>-0.07189914423618531</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7269,7 +7269,7 @@
         <v/>
       </c>
       <c r="D129" s="2" t="n">
-        <v>139.0318218235384</v>
+        <v>139.0318218235383</v>
       </c>
       <c r="E129" s="2" t="n">
         <v>22.1</v>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>53.68369474952561</v>
+        <v>53.68369461291469</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>13.87333230693016</v>
+        <v>13.87333221351431</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.5299852668488549</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>0.2022812343110321</v>
+        <v>0.2022812344346703</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>138.196900864224</v>
+        <v>138.1969008642239</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>16.75</v>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>49.3162773150906</v>
+        <v>49.31627714659567</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>10.93583612762928</v>
+        <v>10.93583615018053</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>1.138483989142189</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>0.0403739946734938</v>
+        <v>0.0403739947147046</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>46.42075684520558</v>
+        <v>46.42075708615643</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>17.75671571590349</v>
+        <v>17.75671562711736</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.2620699716000668</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>0.06966493045861161</v>
+        <v>0.0696649303658842</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>103.3660639017239</v>
+        <v>103.3660639017238</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>11.95</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>47.49013584473407</v>
+        <v>47.49013587577251</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>8.697801117258143</v>
+        <v>8.697801117258138</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.8550479895684145</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.0151791551431053</v>
+        <v>0.0151791551534073</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>97.65693819096629</v>
+        <v>97.65693819096626</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>15.8</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>47.54194864803448</v>
+        <v>47.5419485333363</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>17.28928443111361</v>
+        <v>17.28928450381378</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>0.9211159256646386</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-0.0259362648975487</v>
+        <v>-0.0259362648254288</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>

</xml_diff>